<commit_message>
Add San Pasqual Union ESD district intelligence profile
- Full profile: 548 students, K-8, rural Escondido/San Pasqual Valley
- 11 contacts identified with verified emails (Supt/Principal + 5 board members + staff)
- Board meetings indexed (2025-2026 schedule)
- Science curriculum mapped: 2 STEM teachers, Zoo Safari Park partnership
- 4 vendors/partners with competitive analysis
- Entry strategy targeting Mark Burroughs (Superintendent/Principal)
- Budget pathway: SP School Foundation + Title IV-A (~$3-5K pilot)
- Updated DISTRICT-INTEL-PROMPT.md with validation checklist + small district handling

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/comparison.xlsx
+++ b/comparison.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:Q3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -632,6 +632,87 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>San Pasqual Union ESD</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>San Diego</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>548</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>K-8</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Mark Burroughs</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>16555</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>$9.1M</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>19.87:1</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>36.8%</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>0.9%</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>51.2%</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2.5%</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>23.7%</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>10.4%</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>N/A (K-8)</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Above avg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Q1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -644,7 +725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -785,6 +866,66 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>San Pasqual Union ESD</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>N/A (K-8)</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Est. $300-500K</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Est. $10-15K</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>MS STEM classes, Zoo Safari Park partnership, SAGE Garden</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -797,7 +938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1080,6 +1221,231 @@
         </is>
       </c>
       <c r="I6" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>San Pasqual Union ESD</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Mark Burroughs</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Superintendent/Principal</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>mark.burroughs@sanpasqualunion.net</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>(760) 745-4931 x2300</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>All decisions</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>San Pasqual Union ESD</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Jenny Lynch</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MS STEM Teacher</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>jenny.lynch@sanpasqualunion.net</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>(760) 745-4931</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Teaching</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Classroom champion</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>San Pasqual Union ESD</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Amy Cutchin</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MS STEM Teacher</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>amy.cutchin@sanpasqualunion.net</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>(760) 745-4931</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Teaching</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Classroom champion</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>San Pasqual Union ESD</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Jolene Mallory</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>MS Science Teacher</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>jolene.mallory@sanpasqualunion.net</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>(760) 745-4931</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Teaching</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Science instruction</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>San Pasqual Union ESD</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Kristin DiNofia</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>CBO/Director of Finance</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>kristin.dinofia@sanpasqualunion.net</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>(760) 745-4931</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Business Office</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Budget authority</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1174,7 +1540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1611,6 +1977,194 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>San Pasqual Union ESD</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>San Diego Zoo Safari Park</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Environmental/Science</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Conservation curriculum, applied learning</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>In-kind/TBD</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Deep (long-standing)</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Key differentiator for ModelIt positioning</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>San Pasqual Union ESD</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>S.A.G.E. Garden</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Environmental Ed</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>School garden program</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Volunteer-run</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Community</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Systems modeling opportunity</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>San Pasqual Union ESD</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>SP School Foundation</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Fundraising</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Technology + curriculum funding</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Deep</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Potential pilot funding source</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>San Pasqual Union ESD</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Finalsite</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Website hosting/CMS</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Not competitive</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Website platform only</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1623,7 +2177,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1919,6 +2473,100 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>San Pasqual Union ESD</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>K-5</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>[NEEDS VERIFICATION]</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>San Pasqual Union ESD</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>6-8</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Dedicated STEM + Science teachers</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1931,7 +2579,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2050,6 +2698,58 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>San Pasqual Union ESD</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Mark Burroughs</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Zoo Safari Park + STEM teachers + math gap</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Foundation / Title IV-A</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>$3-5K pilot</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Mar-Jun 2026</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Attend Saints Soiree, send intro email</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Single decision maker, closest to home</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2062,7 +2762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2199,6 +2899,64 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>San Pasqual Union ESD</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Mark Burroughs</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>mark.burroughs@sanpasqualunion.net</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Research complete</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Attend Saints Soiree, send intro email</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>3500</v>
+      </c>
+      <c r="J3" t="n">
+        <v>10000</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Small district, Zoo partnership hook, 15 min from home</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Bear Valley, Lucerne Valley, and Rim of the World district profiles
Three new district intelligence profiles with LCAP analysis, contacts,
entry strategies, and updated comparison spreadsheet and pipeline.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/comparison.xlsx
+++ b/comparison.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:Q7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -794,6 +794,249 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Lucerne Valley USD</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>San Bernardino</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1107</v>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>TK-12</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Peter Livingston</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>22384</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>$22.0M</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>16.82:1</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>57.4%</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>2.3%</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>36.9%</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>0.3%</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>64%</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>~13%</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Red Dashboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Rim of the World USD</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>San Bernardino</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2877</v>
+      </c>
+      <c r="D6" t="n">
+        <v>7</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>K-12</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Dr. Paul Sevillano</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>17591</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>$51.1M</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>22.13:1</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>44.1%</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>0.3%</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>50.6%</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>1.0%</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>39.6%</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>9.0%</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>~86%</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Below avg</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Bear Valley USD</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>San Bernardino</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>2132</v>
+      </c>
+      <c r="D7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>K-12</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Manny Marquez</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>17659</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>$38.3M</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>20.88:1</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>43.1%</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>0.5%</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>49.8%</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>1.0%</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>46.9%</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>~13.6%</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>~86%</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Below avg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Q1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -806,7 +1049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1067,6 +1310,188 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Lucerne Valley USD</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>$700K (2yr CTE)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Est. $2-3M</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Est. $300-500K</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Est. $15-25K</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>8</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Bud Biggs STEM Lab, FFA, DI, Future City, CTE 80%+ participation</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Rim of the World USD</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Construction/Fire/Auto/TV</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Est. $5.3M</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>4</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Renewable energy (solar+wind), Robotics, FFA, AVID</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Bear Valley USD</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>BEARTECH, STEAM Nights, AVID, dual enrollment</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1079,7 +1504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1633,6 +2058,546 @@
       </c>
       <c r="I12" t="n">
         <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Lucerne Valley USD</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Peter Livingston</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Superintendent</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>peter_livingston@lucernevalleyusd.org</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>(760) 248-6108 x4131</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Final authority</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Yes (BestNet President)</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Lucerne Valley USD</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Aaron Jones</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Director of Academic Programs</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>aaron_jones@lucernevalleyusd.org [INFERRED]</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Curriculum</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Primary curriculum buyer</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Indirect</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Lucerne Valley USD</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Jessica Haecker</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CTE Coordinator / Asst. Principal</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>jessica_haecker@lucernevalleyusd.org [INFERRED]</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>CTE</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>CTE integration</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Lucerne Valley USD</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Olga Fisher</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Asst. Supt. Business Services</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>olga_fisher@lucernevalleyusd.org</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Budget authority</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Rim of the World USD</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Dr. Paul Sevillano</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Superintendent</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>paul_sevillano@rimsd.k12.ca.us</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>(909) 336-4100 x105</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Final authority</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Indirect</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Rim of the World USD</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Jennifer Whiteside</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Director of Educational Services</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>jennifer_whiteside@rimsd.k12.ca.us [INFERRED]</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Curriculum</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Curriculum gatekeeper</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Indirect</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Rim of the World USD</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Stephanie Phillips</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CTE/ROP Coordinator</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>stephanie_phillips@rimsd.k12.ca.us</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>(909) 336-2038 x282</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>CTE</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>CTE integration</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Rim of the World USD</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Jordana Ridland</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Board Member</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>jordana_ridland@rimsd.k12.ca.us</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Board</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Board champion</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Yes (former math teacher, MA Ed Tech)</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Bear Valley USD</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Manny Marquez</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Superintendent</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>manny_marquez@bearvalleyusd.org</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>(909) 866-4631</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Final authority</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Indirect</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Bear Valley USD</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Leigh Anne Drake</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Exec. Dir. TK-6 Curriculum</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>leighanne_drake@bearvalleyusd.org</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Curriculum</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Elementary curriculum buyer</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Indirect</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Bear Valley USD</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Brian Willemse</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Exec. Dir. 6-12 Curriculum</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>brian_willemse@bearvalleyusd.org</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Curriculum</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>6-12 curriculum buyer</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Indirect</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Bear Valley USD</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Dr. Stephen Foulkes</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Board President</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>steve_foulkes@bearvalleyusd.org</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Board</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Board champion</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Yes (PhD Physics)</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -1726,7 +2691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2439,7 +3404,545 @@
           <t>Vendor</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Lucerne Valley USD</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Victor Valley College</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Higher Ed</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Dual enrollment Ag courses</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Not competitive</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Deep</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>On-site college courses</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Lucerne Valley USD</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Mitsubishi Cement / Ed Foundation</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Industry</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Field trips, Foundation board</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Not competitive</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Deep</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Supt on Foundation board</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Lucerne Valley USD</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>BestNet JPA</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>County tech consortium</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Not competitive</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Deep</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Supt is President</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Lucerne Valley USD</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Victor HS District</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>CTE Funding</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>$380K CTE partnership</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>$380K</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Multi-year</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Not competitive</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Deep</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Major CTE funder</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Rim of the World USD</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>ParentSquare</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Family communication</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Not competitive</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Rim of the World USD</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Care Solace</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Mental health referral service</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Not competitive</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Rim of the World USD</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Rim Educational Foundation</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Fundraising</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>AVID, CTE/ROP, school grants</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Since 1983</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Deep</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Funds CTE since 2015</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Rim of the World USD</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>tBP Architecture</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Construction</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Measure E bond projects</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Part of $71M</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Multi-year</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Not competitive</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Bear Valley USD</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Big Bear Valley Ed Trust</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Community</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>BEARTECH, STEMQUEST, Pebble Plain</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Deep</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Key STEM partner</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Bear Valley USD</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>BVUSD Education Foundation</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Fundraising</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>213-acre outdoor ed property</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Deep</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Outdoor education</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Bear Valley USD</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>San Bernardino Valley College</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Higher Ed</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Dual enrollment at Big Bear Mountain Center</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Not competitive</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Bear Valley USD</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ParentSquare / StudentSquare</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Family communication</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Not competitive</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
@@ -2453,7 +3956,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2984,6 +4487,382 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Lucerne Valley USD</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>K-6</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Bud Biggs STEM Lab supplements instruction</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Lucerne Valley USD</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>7-12</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>TBD (incl. Ag Biology)</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>FFA program with Ag Bio; dual enrollment with VVC</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Rim of the World USD</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>K-5</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>3 elementary schools</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Rim of the World USD</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>6-8</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Mary Putnam Henck Intermediate</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Rim of the World USD</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>9-12</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>4 science teachers at Rim High; renewable energy project</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Bear Valley USD</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>K-5</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>BEARTECH program at elementary</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Bear Valley USD</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>6-8</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Big Bear Middle School</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Bear Valley USD</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>9-12</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>McKenzie Wolf is Science Dept lead</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2996,7 +4875,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3219,6 +5098,162 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Lucerne Valley USD</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Aaron Jones</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>STEM Lab + FFA + CTE + 10.69% math crisis</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Title I + CSI + CTE grants</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>$5-10K pilot</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Feb-Jun 2026</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Email intro re: Dashboard recovery</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Feb-Mar 2026</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>New academic director in buying mode; red Dashboard; CTE 80% participation</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Rim of the World USD</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Jennifer Whiteside</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Mountain ecology + renewable energy + math gap + Measure E</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>LCFF Supp/Conc + Measure E</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>$10-15K pilot</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Mar-Jun 2026</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Email intro re: math gap + Measure E</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Former math teacher on board; $71M bond; renewable energy pioneer</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Bear Valley USD</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Leigh Anne Drake</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>BEARTECH + mountain ecology + Physics PhD board president</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>LCFF Supp/Conc + Title I</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>$5-10K pilot</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Mar-Jun 2026</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Email intro re: BEARTECH + math gap</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Board president has PhD Physics; BEARTECH nature-based STEM program</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3231,7 +5266,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3484,6 +5519,180 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Lucerne Valley USD</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Aaron Jones</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>aaron_jones@lucernevalleyusd.org [INFERRED]</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Research complete</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Email intro re: Dashboard recovery</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-02-15</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>5000</v>
+      </c>
+      <c r="J5" t="n">
+        <v>15000</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Red Dashboard, new academic director, CTE 80%, STEM Lab, 2hr from Carlsbad</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Rim of the World USD</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Jennifer Whiteside</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>jennifer_whiteside@rimsd.k12.ca.us [INFERRED]</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Research complete</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Email intro re: math gap + Measure E</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J6" t="n">
+        <v>30000</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>$71M bond, renewable energy, mountain ecology, Ed Foundation</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Bear Valley USD</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Leigh Anne Drake</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>leighanne_drake@bearvalleyusd.org</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Research complete</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Email intro re: BEARTECH + math gap</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>5000</v>
+      </c>
+      <c r="J7" t="n">
+        <v>15000</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Physics PhD board president, BEARTECH, 213-acre outdoor ed property</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add La Habra City SD district intelligence profile
- Full profile with demographics, test scores, STEM programs (K-8, 4,244 students)
- 7 contacts identified; emails not publicly listed (use Contact Us form)
- Board meetings indexed (2025-present)
- Science curriculum mapped by grade band; PLTW Gateway confirmed at middle schools
- 6 vendors/partners with competitive analysis
- Entry strategy targeting Dr. Patricia Sandoval (Asst. Supt. of Ed Services)
- Budget pathway: LCFF Supp/Conc + Title I + Title III (bilingual)
- Key hooks: $73M Measure O bond, STEAM Academies, 86% Hispanic, 11.78% EL math

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/comparison.xlsx
+++ b/comparison.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1037,6 +1037,87 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>La Habra City SD</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>4244</v>
+      </c>
+      <c r="D8" t="n">
+        <v>9</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>K-8</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Dr. Mario A. Carlos, Ed.D.</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>16186</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>~$81.9M</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>86.2%</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>0.9%</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>6.9%</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>3.7%</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>80.3%</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>20.6%</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>N/A (K-8)</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Average</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Q1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1049,7 +1130,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1492,6 +1573,68 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>La Habra City SD</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>N/A (K-8)</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>TBD (est. $10-15M)</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>TBD (est. $1.5-3M)</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Science &amp; Tech Academy (2), PLTW Gateway, robotics clubs, 1:1 devices, $73M Measure O bond</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1504,7 +1647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2598,6 +2741,231 @@
       </c>
       <c r="I24" t="n">
         <v>4</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>La Habra City SD</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Dr. Patricia Sandoval</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Asst. Superintendent of Educational Services</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>(562) 690-2305</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Educational Services</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Primary decision maker</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Possible (Innovative Ed background)</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>La Habra City SD</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Dr. Mario A. Carlos, Ed.D.</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Superintendent</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>(562) 690-2305</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Final authority</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>La Habra City SD</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Emily Flesher</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Director of Special Programs &amp; Assessment</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Educational Services</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Assessment &amp; categorical funding</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>La Habra City SD</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Anna Navarro</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Program Specialist / Multilingual Support</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Educational Services</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>EL champion</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Yes (bilingual connection)</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>La Habra City SD</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Jody Green</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Academic Coach</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Educational Services</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Classroom influencer</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Possible</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -2691,7 +3059,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I27"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3944,6 +4312,284 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>La Habra City SD</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Project Lead the Way (PLTW)</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>STEM Curriculum</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Gateway modules (design, robotics, coding, CS)</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>At middle schools</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>La Habra City SD</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Boys &amp; Girls Club of La Habra</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Community Partner</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>ELO-P after-school STEM enrichment</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Not competitive</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Robotics clubs</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>La Habra City SD</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>CampusSuite/Finalsite</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Website hosting/CMS</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Not competitive</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>La Habra City SD</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Chromebooks / Google Workspace</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Not competitive</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>1:1 Chromebooks grades 2-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>La Habra City SD</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Apple</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>iPads</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Not competitive</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>600+ iPads at middle schools</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>La Habra City SD</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Cal Poly Pomona</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Higher Ed</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Robotics competition connection</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Not competitive</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Student competition destination</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3956,7 +4602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4863,6 +5509,100 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>La Habra City SD</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>K-6</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Core curriculum</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>[NEEDS VERIFICATION] Science &amp; Tech Academy at Walnut Elem</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>La Habra City SD</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>6-8</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Core curriculum</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>[NEEDS VERIFICATION] PLTW Gateway supplements at middle schools</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4875,7 +5615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5254,6 +5994,58 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>La Habra City SD</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Dr. Patricia Sandoval</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>STEAM Academies + $73M Measure O + 86% Hispanic + 11.78% EL math</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>LCFF Supp/Conc + Title I + Title III</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>$10-15K pilot</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Mar-Jun 2026</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Phone call to district office, request meeting</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>K-8 district; new Ed Services leader (Jan 2024); PLTW complement angle; bilingual emphasis</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5266,7 +6058,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5693,6 +6485,64 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>La Habra City SD</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Dr. Patricia Sandoval</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Research complete</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Phone call to district office</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J8" t="n">
+        <v>40000</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>$73M Measure O, STEAM Academies, PLTW, 86% Hispanic, 80% ED, 21% EL</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Valley Center-Pauma USD district intelligence profile
- Full profile with demographics, test scores (18% math, 29% ELA, 19% science), STEM programs
- 5+ contacts identified (Superintendent Hailwood [new Jan 2026], AP Clymer, HR Rogers, Howard)
- Board meetings indexed via BoardDocs portal
- Science curriculum mapped: Agriculture/FFA flagship, ForeFront Power STEAM integration
- 7+ vendors/partners: CSUSM, ForeFront Power solar, Rincon/Pauma tribal MOUs, Palomar College
- Entry strategy targeting Mark Hailwood (new superintendent with explicit math instruction priority)
- Budget pathway: LCFF Supplemental/Concentration + Title I ($10-15K pilot)
- Unique hooks: agriculture modeling, bilingual Dual Immersion, solar STEAM extension, tribal partnerships

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/comparison.xlsx
+++ b/comparison.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q8"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1118,6 +1118,79 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Valley Center-Pauma USD</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>San Diego</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>3636</v>
+      </c>
+      <c r="D9" t="n">
+        <v>8</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>K-12</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Mark Hailwood</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>15305</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>$58M</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>22:1</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>63%</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>20.6%</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>43.8%</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>24.2%</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>94%</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Rural; Math 18%, ELA 29%, Sci 19%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Q1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1130,7 +1203,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1635,6 +1708,68 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Valley Center-Pauma USD</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>CTEIG/Perkins (expanding)</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Est. $5-8M</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Est. $500K-1M</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Agriculture/FFA, Media Technology</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Agriculture/FFA, Media Tech CTE, ForeFront Power STEAM, Dual Immersion</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1647,7 +1782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2966,6 +3101,207 @@
       </c>
       <c r="I29" t="n">
         <v>5</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Valley Center-Pauma USD</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Mark Hailwood</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Superintendent</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>hailwood.ma@vcpusd.org</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Administration</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Final decision maker</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Valley Center-Pauma USD</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Nicole Clymer</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>AP VCHS</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>clymer.ni@vcpusd.org</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Site Admin</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>HS instructional lead</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Valley Center-Pauma USD</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Aaron Rogers</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Asst Supt HR</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>rogers.aa@vcpusd.org</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Human Resources</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>HR/staffing support</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Valley Center-Pauma USD</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Doyan Howard</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Dir Student Support Services</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>howard.do@vcpusd.org</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Student Services</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Student support programs</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Valley Center-Pauma USD</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Ed Services Director</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Education Services</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Curriculum decisions</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -3059,7 +3395,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4447,7 +4783,6 @@
           <t>Vendor</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -4587,6 +4922,335 @@
       <c r="I33" t="inlineStr">
         <is>
           <t>Student competition destination</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Valley Center-Pauma USD</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>ForeFront Power</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>STEAM Partner</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Solar/STEAM educational program</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Active partnership</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Solar STEAM program at schools</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Valley Center-Pauma USD</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>CSUSM</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Higher Ed</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Partnership for Success program</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Institutional partnership</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>College readiness pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Valley Center-Pauma USD</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Rincon Band</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Tribal MOU</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Tribal community partnership</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>MOU</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Tribal education/cultural partnership</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Valley Center-Pauma USD</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Pauma Band</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Community</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Community partnership</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Community relationship</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Tribal community engagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Valley Center-Pauma USD</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Palomar College</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Higher Ed</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Dual enrollment / higher ed pipeline</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Partnership</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>College pathways for HS students</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Valley Center-Pauma USD</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Finalsite</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>District website platform</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Vendor contract</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Website/CMS provider</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Valley Center-Pauma USD</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>BoardDocs</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Board meeting management</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Vendor contract</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Board agenda/minutes platform</t>
         </is>
       </c>
     </row>
@@ -4602,7 +5266,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5603,6 +6267,194 @@
         </is>
       </c>
     </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Valley Center-Pauma USD</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>K-5</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Needs research</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Valley Center-Pauma USD</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>6-8</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Needs research</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Valley Center-Pauma USD</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>9-12</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Agriculture Biology (FFA)</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>CTE/Science</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>FFA agriculture biology + general science courses</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Valley Center-Pauma USD</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>K-12 Supplemental</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>ForeFront Power STEAM</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Supplemental/STEAM</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Solar STEAM program; also Dual Immersion (EN/ES)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5615,7 +6467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6046,6 +6898,58 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Valley Center-Pauma USD</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Mark Hailwood (Superintendent)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Math priority + agriculture modeling + bilingual + solar STEAM</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>LCFF Supp/Conc + Title I</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>$10-15K pilot</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Feb-Jun 2026 LCAP cycle</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Email intro to Hailwood re: math priority + agriculture</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Feb-Mar 2026</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Rural district, 63% Hispanic, agriculture/FFA focus, tribal partnerships, 24% EL, low math proficiency (18%)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6058,7 +6962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6543,6 +7447,64 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Valley Center-Pauma USD</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Mark Hailwood</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>hailwood.ma@vcpusd.org</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Research complete</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Email intro to Hailwood re: math priority + agriculture</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>12500</v>
+      </c>
+      <c r="J9" t="n">
+        <v>25000</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>$10-15K pilot -&gt; $25K scale; rural, agriculture/FFA, bilingual, tribal, low math 18%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Fountain Valley SD district intelligence profile
- Full profile: 6,022 students, K-8, Orange County, 74% math proficiency
- 9 contacts identified (5 board emails verified from fvsd.us)
- Board meetings indexed (2025-2026), purchasing/warrant tracking added
- Science curriculum mapped: Discovery Ed (K-5), Amplify (6-8)
- 12 vendors/partners with competitive analysis (no direct competitors)
- Entry strategy targeting Dr. Jerry Gargus (Asst. Supt. Ed Services)
- Budget pathway: LCFF S&C ($50-100K) + General Fund ($30-50K)
- Enrichment positioning for high-performing district with equity gaps
- Pipeline updated: 10 districts, $113K-590K total value
- Comparison spreadsheet updated across all 8 sheets

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/comparison.xlsx
+++ b/comparison.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q10"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1270,6 +1270,93 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Orange</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>6022</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>K-8</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Dr. Katherine Stopp, Ed.D.</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>11571</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>~$112M</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>19.2%</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>32.1%</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>37.5%</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>23.6%</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>~10%</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>N/A (K-8)</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Strong; Math 74.04%, ELA 78.71%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Q1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1282,7 +1369,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1911,6 +1998,68 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>N/A (K-8)</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>~$3.2M</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>TBD (4 schools qualify: Cox, Masuda, Oka, Plavan)</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>N/A (K-8)</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Robotics (all schools), ENGIE Living Labs, Measure O Bond ($63M), ENGIE savings ($6.8M lifetime), Strong local tax base (55% of revenue)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1923,7 +2072,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3797,6 +3946,241 @@
       </c>
       <c r="I42" t="n">
         <v>2</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Dr. Jerry Gargus, Ed.D.</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Asst. Superintendent of Ed Services</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Education Services</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>STEM program selection &amp; curriculum approval</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Dr. Kiva Spiratos, Ed.D.</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Director of Ed Services</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>kspiratos@fvsd.us</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Education Services</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Curriculum &amp; instruction oversight</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Dr. Katherine Stopp, Ed.D.</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Superintendent</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Superintendent's Office</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Executive approval</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Dennis Cole</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Board President</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>denniscole@fvsd.us</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Board of Education</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Board champion; OCDE Chief of Staff</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Ashley Ramirez</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Board Member</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>ramirezashley@fvsd.us</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Board of Education</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Innovation advocate; UCI Innovation</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3890,7 +4274,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6266,6 +6650,617 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Discovery Education</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Curriculum</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>K-5 Science (CA Science)</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>2020-present</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Annual contract</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>Primary K-5 science platform</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Amplify</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Curriculum</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>6-8 Science (CA Science Program)</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>2020-present</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Annual contract</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>Primary 6-8 science platform</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>HMH Math Expressions</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Curriculum</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>K-5 Math</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>2020-present</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Annual contract</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>Primary K-5 math program</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>McGraw Hill CA Math</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Curriculum</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>6-8 Math</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>2016-present</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Annual contract</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>Older adoption; may be due for refresh</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>1:1 Chromebooks</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Deep integration</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>District-wide 1:1 program</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Clever</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>SSO platform</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Annual contract</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>Single sign-on for all ed-tech</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Aeries</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Student Information System (SIS)</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>Deep integration</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>Primary SIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>IXL</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Curriculum</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Math &amp; ELA practice</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>Annual contract</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>Supplemental</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Khan Academy</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Curriculum</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Math &amp; general enrichment</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>Supplemental</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>Free resource</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Desmos</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Curriculum</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Math graphing &amp; activities</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Free</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>Supplemental</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>Free resource</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>BrainPOP</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Curriculum</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Animated science/math lessons</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>Annual contract</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>Supplemental across subjects</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>ENGIE</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Living Labs sustainability program</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Part of $6.8M savings</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>Strategic partner</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>ENGIE Living Labs at school sites</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Diligent (BoardDocs)</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Board meeting management</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>Annual contract</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>BoardDocs for agenda/minutes</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6278,7 +7273,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7702,6 +8697,288 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>K-5</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Discovery Education California Science</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Digital Platform</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Primary K-5 science curriculum</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>6-8</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Amplify CA Science Program</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Digital Platform</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Primary 6-8 science curriculum</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>K-8</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Robotics programs</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Supplemental</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Available at all schools</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>K-8</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>ENGIE Living Labs</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Supplemental</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Sustainability/environmental science</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>K-8</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>BrainPOP</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Digital Lessons</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Supplemental animated lessons</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>K-8</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>1:1 Chromebooks (Google)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Device infrastructure for all digital programs</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7714,7 +8991,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8249,6 +9526,58 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Dr. Jerry Gargus, Ed.D.</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>74% math is excellent, but Hispanic at 57%, EL at 43%. Math drops from 85% to 68% in middle school. NGSS Practice 2 enrichment + equity.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>LCFF S&amp;C ($50-100K) + General Fund ($30-50K)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>$50-100K</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>LCAP cycle 2026</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Email intro via district office</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Suburban Orange County, strong tax base, Measure O bond ($63M), ENGIE partnership, K-8 only</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8261,7 +9590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8862,6 +10191,68 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Fountain Valley SD</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Dr. Jerry Gargus, Ed.D.</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Research complete</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Email intro via district office</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>50000</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>K-8 suburban OC, 74% math proficiency, equity gap (Hispanic 57%, EL 43%), Measure O $63M bond, ENGIE Living Labs</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Carlsbad Unified district intelligence profile
- Full profile: 10,982 students, San Diego County, K-12, Priority 35/100
- 8 contacts identified with verified emails (Ashley Crawford primary)
- Board meetings indexed 2025-present (22 meetings with PDF links)
- Science curriculum mapped: PLTW at Calavera Hills MS + Sage Creek HS
- 14 vendors/partners identified (PLTW, CEF, Viasat, AHLF, Google, Renaissance, etc.)
- Entry strategy: STEAM labs + EL science gap (19.2%) + new Supt hook
- Budget pathway: Instructional materials + Title IV-A + CEF co-funding
- Primary contact: Ashley Crawford (acrawford@carlsbadusd.net)
- comparison.xlsx updated (all 8 sheets)
- pipeline.md updated (15 districts total)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/comparison.xlsx
+++ b/comparison.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:Q12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1357,6 +1357,87 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>San Diego</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>10982</v>
+      </c>
+      <c r="D12" t="n">
+        <v>16</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>K-12</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Dr. Andrea Norman</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>13879</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>$172.8M</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>22.4:1</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>26.3%</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>1.4%</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>55.5%</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>5.3%</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>4.7%</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>4.6%</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>~95%</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>A+ (Niche)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Q1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1369,7 +1450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2060,6 +2141,48 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>$200K+ (CEF) + Measure HH</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>TBD [NEEDS VERIFICATION]</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Part of $265M Measure HH</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>PLTW + Perkins IV</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>$6,572,669</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2072,7 +2195,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4178,6 +4301,241 @@
         </is>
       </c>
       <c r="I47" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Ashley Crawford</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>K-12 Science Specialist / TOSA</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>acrawford@carlsbadusd.net</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>(760) 331-5059</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Instructional Services</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Science curriculum evaluator</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Nicole Moersch</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>K-12 CTE Specialist</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>nmoersch@carlsbadusd.net</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>(760) 331-5040</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Instructional Services</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>CTE/PLTW decision-maker</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Bryan Brockett</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Asst. Superintendent, Instructional Services</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>bbrockett@carlsbadusd.net</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>(760) 331-5013</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Instructional Services</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Budget authority / approver</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>John Moreno</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>K-12 Math Specialist / TOSA</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>jmoreno@carlsbadusd.net</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>(760) 331-5034</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Instructional Services</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Math curriculum evaluator</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Robert Allen</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Director, Assessment &amp; Technology</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>its@carlsbadusd.net</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>(760) 331-5000</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>IT/Technology</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>EdTech approval / data privacy</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
         <is>
           <t>5</t>
         </is>
@@ -4274,7 +4632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7261,6 +7619,436 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Project Lead the Way (PLTW)</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Curriculum</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>K-12 STEM pathway courses</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Deep - multi-year</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Renaissance Learning (STAR)</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Reading + math screener Gr1-12</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>Annual contract</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Amplify (DIBELS 8)</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>K-2 literacy screener</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>Annual contract</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Achieve3000</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>EdTech</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Differentiated reading platform</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>Annual contract</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Google (Workspace/Chromebooks)</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>1:1 devices, LMS, AI tools</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Core infrastructure</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>MagicSchool AI</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>EdTech/AI</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>AI adaptive quizzes</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Active (recently adopted)</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>New tool</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Snorkl AI</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>EdTech/AI</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Student work analysis / feedback</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Active (recently adopted)</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>New tool</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Carlsbad Educational Foundation (CEF)</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Community Partner</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>STEM funding: robotics, STEAM, Science Olympiad</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>$200K+/yr STEM</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Deep - primary funder</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Agua Hedionda Lagoon Foundation</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Environmental Partner</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Gr3+7 field trips; NGSS water sampling</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Program partner</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Viasat</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Industry Partner</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>8-yr Science Olympiad sponsor; employee mentors</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Active 8+ years</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Sponsor</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7273,7 +8061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -8979,6 +9767,147 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>K-5</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>TBD - Not publicly confirmed</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Expected Yes</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>[NEEDS VERIFICATION] - Contact Ashley Crawford</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>6-8</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>PLTW modules (Energy+Env, Medical Det, Design) + TBD mainstream</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Yes (PLTW)</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Calavera Hills is PLTW hub; mainstream publisher TBD</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>9-12</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>PLTW Engineering + Biomedical (Sage Creek); Glencoe Biology (alt.)</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Sage Creek PLTW Distinguished 2022</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -8991,7 +9920,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9578,6 +10507,48 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Ashley Crawford (Science TOSA)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>STEAM Labs + EL science gap (19.2%) + NGSS SEP-2 modeling missing link</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>LCFF Supplemental (EL) + Instructional Materials budget</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>$10-25K pilot / $50K+ district</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>March-June 2026</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Send intro email to Ashley Crawford</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9590,7 +10561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10253,6 +11224,48 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Ashley Crawford</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>acrawford@carlsbadusd.net</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Research complete</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Send intro email + demo request</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Enhance Carlsbad Unified district intelligence profile
- Fully rewrote entry-strategy.md: 5-phase approach, 10 risks, key dates calendar
- Fully rewrote pitch-notes.md: 2 email templates, 7 talking points, 8 objection responses
- Fully rewrote science-curriculum.md: PLTW positioning matrix, grade-band priority, competitor analysis
- Fully rewrote vendors-partners.md: complete vendor map, warm intro paths, competitive risk table
- Updated comparison.xlsx: all 8 sheets refreshed with Carlsbad USD data
- Primary contact: Ashley Crawford (K-12 Science TOSA)
- Hook: PLTW STEAM Labs + EL science 19.2% gap + bilingual

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/comparison.xlsx
+++ b/comparison.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q12"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1438,6 +1438,87 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>San Diego</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>10982</v>
+      </c>
+      <c r="D13" t="n">
+        <v>16</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>TK-12</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Dr. Andrea Norman</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>13879</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>~$133.3M</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>22:1</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>26.3%</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>1.4%</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>55.5%</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>5.3%</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>4.7%</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>4.6%</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>~95%</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>A+ (Niche)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Q1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1450,7 +1531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2183,6 +2264,68 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Minimal (&lt;1M est, 4.7% SED)</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Limited (low poverty)</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>~$50-100K est.</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>12 (HS pathways)</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>PLTW K-12, STEAM Labs, FIRST, Robotics, Science Days, Science Olympiad</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2195,7 +2338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4539,6 +4682,231 @@
         <is>
           <t>5</t>
         </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Ashley Crawford</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>K-12 Science Specialist/TOSA</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>acrawford@carlsbadusd.net (inferred)</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>(760) 331-5013</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Instructional Services</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>First recommender for science tools</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Dr. Bryan Brockett</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Asst. Supt. Instructional Services</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>bbrockett@carlsbadusd.net</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>(760) 331-5013</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>District Office</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Budget approval for curriculum tools</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Nicole Moersch</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>K-12 CTE/PLTW Specialist/TOSA</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>nmoersch@carlsbadusd.net (inferred)</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>(760) 331-5013</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Instructional Services</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>PLTW and CTE program decisions</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Joseph Hartman</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Director Assessment &amp; Technology</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>jhartman@carlsbadusd.net (inferred)</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>(760) 331-5000</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>IT/Assessment</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>EdTech adoption; Title IV-A budget</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Dr. Andrea Norman</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Superintendent</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>andrea.norman@carlsbadusd.net</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>(760) 331-5001</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>District Office</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Final budget authority; new June 2025</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -4632,7 +5000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:I82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7660,7 +8028,6 @@
           <t>Deep - multi-year</t>
         </is>
       </c>
-      <c r="I65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -7703,7 +8070,6 @@
           <t>Annual contract</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -7746,7 +8112,6 @@
           <t>Annual contract</t>
         </is>
       </c>
-      <c r="I67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -7789,7 +8154,6 @@
           <t>Annual contract</t>
         </is>
       </c>
-      <c r="I68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -7832,7 +8196,6 @@
           <t>Core infrastructure</t>
         </is>
       </c>
-      <c r="I69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -7875,7 +8238,6 @@
           <t>New tool</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -7918,7 +8280,6 @@
           <t>New tool</t>
         </is>
       </c>
-      <c r="I71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -7961,7 +8322,6 @@
           <t>Deep - primary funder</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -8004,7 +8364,6 @@
           <t>Program partner</t>
         </is>
       </c>
-      <c r="I73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -8047,7 +8406,382 @@
           <t>Sponsor</t>
         </is>
       </c>
-      <c r="I74" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Project Lead the Way (PLTW)</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Curriculum</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>K-12 STEM pathway (Engineering, Biomedical, CS, Elementary)</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>District partner</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>PLTW Distinguished 2022 at Sage Creek HS</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Renaissance Learning (STAR)</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Universal screener math+reading Grades 1-12</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>No - different use</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>Annual contract</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>District-wide</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Amplify (DIBELS 8th Ed)</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Assessment</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Early literacy K-2</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>No - different use</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>Annual contract</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>K-2 only</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Achieve3000</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>EdTech</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Differentiated reading platform</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>No - different use</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>Annual contract</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>District-wide</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Google Workspace for Education</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>LMS/Ecosystem</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Primary productivity + LMS + Gemini AI</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>District ecosystem</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>All-in Google district</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Snorkl</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>AI Tools</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>AI student work analysis and feedback</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>New adoption 2024-25</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>Active use</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>VEX Robotics</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>STEM Hardware</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Robotics platform Grade 6 (Calavera Hills MS)</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>PLTW partnership</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>PLTW Automation &amp; Robotics</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Carlsbad Educational Foundation</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Community Partner</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Funds: STEAM, robotics, FIRST, Science Days, field trips</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Grants</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>Deep - primary funder</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Key relationship for grant pathway</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
@@ -8061,7 +8795,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9908,6 +10642,147 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>K-5</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>TBD - needs verification</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Core + Supplemental PLTW</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Contact Ashley Crawford; STEAM Labs being built at 8 elementaries</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>6-8</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>TBD - needs verification</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Core + PLTW: Automation, Energy, Medical Detectives, Design</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Calavera Hills MS: full PLTW STEM pathway</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>9-12</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>TBD - needs verification</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Core + PLTW Engineering (4-course) + PLTW Biomedical (4-course)</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Sage Creek: PLTW Distinguished 2022</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9920,7 +10795,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10549,6 +11424,58 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Ashley Crawford (K-12 Science TOSA)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>PLTW STEAM Labs + EL science 19.2% gap + bilingual + NGSS SEP 2+5</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Measure HH Bond / Title IV-A / Site Discretionary</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>$5-15K pilot</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>April-June 2026 (LCAP window)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Verify email, send intro email</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>March 2026</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>High-performing enrichment play; EL equity subgroup angle; new supt June 2025</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10561,7 +11488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11266,6 +12193,64 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Carlsbad USD</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Ashley Crawford</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>acrawford@carlsbadusd.net (inferred)</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Research complete</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Verify email, send intro email</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J13" t="n">
+        <v>40000</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>High-performing enrichment play; PLTW hook; EL science 19.2%; Measure HH STEAM Labs; new supt</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Arvin Union ESD district intelligence profile
- Full profile with demographics, CAASPP/CAST test scores, STEM programs
- 25 contacts identified across 5 tiers with wave outreach plan
- Board meetings indexed (2025-present); eBoard/Simbli portal documented
- Science curriculum: NO confirmed vendor = complete white space (primary hook)
- 8 vendors/partners mapped; Canvas + Clever + i-Ready confirmed
- Entry strategy: Kerrie Nisser (Director C&I) as primary, Title IV-A pathway
- Budget pathway: Title IV-A (SSAE) + LCFF Supplemental (~$12-25K pilot)
- Bilingual platform fit: 15.5% EL + Dual Immersion program
- Priority score: 95/100 (Kern County, 15.71% CAST, greenfield science)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/comparison.xlsx
+++ b/comparison.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q15"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1681,6 +1681,87 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Arvin Union ESD</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Kern</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2963</v>
+      </c>
+      <c r="D16" t="n">
+        <v>4</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>TK-8</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Georgia Rhett</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>18102</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>$64.3M</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>92.8%</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>0.8%</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>5.8%</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>~94% (FRPM)</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>15.5%</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>N/A (elem dist)</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Q1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1693,7 +1774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2608,6 +2689,68 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Arvin Union ESD</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>None confirmed</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>i-Ready (Curriculum Assoc.)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Chromebooks + Canvas</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>N/A (elem dist)</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Est. $10-12M (LCFF Supp/Conc)</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Est. $3-4M</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Est. $50-150K</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>AVID schoolwide; Dual Immersion; Expanded Learning (ASES)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2620,7 +2763,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5516,6 +5659,231 @@
         </is>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Arvin Union ESD</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Kerrie Nisser</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Director of Curriculum, Instruction &amp; Assessment</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>knisser@arvin-do.com</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>(661) 854-6518</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Curriculum &amp; Instruction</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Controls curriculum adoption and EdTech selection</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Arvin Union ESD</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Georgia Rhett</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Superintendent</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>grhett@arvin-do.com</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>(661) 854-6500</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>District Office</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Final budget authority</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Arvin Union ESD</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Larry Horton</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>District TOSA &amp; AVID Director</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>lhorton@arvin-do.com</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>(661) 854-6500</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Curriculum &amp; Instruction</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>TOSA implementation champion</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Arvin Union ESD</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Magdalena Hernandez</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Principal, Haven Drive Middle School</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>mhernandez@arvin-do.com</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>(661) 854-6540</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Site Leadership</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Grade 8 CAST pilot site champion</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Arvin Union ESD</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Chris Davis</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Chief Business Official</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>cdavis@arvin-do.com</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>(661) 854-6500</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Business Office</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Controls Title IV-A and federal budget codes</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5528,7 +5896,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5647,6 +6015,58 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Arvin Union ESD</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Science curriculum adoption (unknown vendor)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Curriculum</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>LCFF Supplemental / Title I</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>eBoard/Simbli - arvinschools.com/board</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Needs board minutes PDF review</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5659,7 +6079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I97"/>
+  <dimension ref="A1:I103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10147,6 +10567,288 @@
         </is>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Arvin Union ESD</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Curriculum Associates (i-Ready)</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>EdTech</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Math/reading diagnostic + instruction</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>Math/reading covered; science is open white space</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Arvin Union ESD</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Instructure (Canvas)</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>LMS</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>Learning Management System</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>ModelIt embeds in Canvas; zero integration friction</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Arvin Union ESD</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Clever</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>SSO</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>Student Single Sign-On portal</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>ModelIt can use Clever SSO; no new student login</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Arvin Union ESD</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>AVID Center</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>PD/Curriculum</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>College readiness program</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Confirmed</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>Schoolwide AVID; Larry Horton = AVID Director</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Arvin Union ESD</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Google (Workspace)</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Productivity</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Google Forms, Docs, Drive</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Likely</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>Google Forms confirmed for afterschool registration</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Arvin Union ESD</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Science vendor</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Curriculum</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>NGSS science program</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Complementary</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>NO confirmed science publisher — complete white space for ModelIt</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10159,7 +10861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I46"/>
+  <dimension ref="A1:I49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12335,6 +13037,147 @@
         </is>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Arvin Union ESD</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>K-5 (Elem)</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>UNKNOWN — no confirmed publisher</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>No NGSS-aligned curriculum confirmed; call Kerrie Nisser to verify</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Arvin Union ESD</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>6-8 (Middle)</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>UNKNOWN — no confirmed publisher</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Haven Drive MS (Gr.7-8) is CAST pilot target; science curriculum unknown</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Arvin Union ESD</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>9-12</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>N/A — elementary district</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Elementary district only (TK-8); no high school</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -12347,7 +13190,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13132,6 +13975,58 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Arvin Union ESD</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Kerrie Nisser (Director C&amp;I)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>15.71% CAST + no confirmed science vendor + Canvas/Clever integration + 59% Nearly Met cohort</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Title IV-A (SSAE) / LCFF Supplemental</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>$12-25K pilot → $40-60K district-wide</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Mar-Jun 2026 (LCAP window)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Send intro email to Kerrie Nisser + Larry Horton</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Mar 2026</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Bilingual platform fit; zero integration; science is lowest subject with no vendor</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -13144,7 +14039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14023,6 +14918,64 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Arvin Union ESD</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Kerrie Nisser</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>knisser@arvin-do.com</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Research complete</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Send intro email</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>12000</v>
+      </c>
+      <c r="J16" t="n">
+        <v>60000</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>25%</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>15.71% CAST; no science vendor; Canvas+Clever ready; Title IV-A pathway; bilingual fit</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Beardsley Elementary School District intelligence profile
- Full profile with demographics, test scores, STEM programs
- 30 contacts identified with verified dept email + inferred pattern
- PLTW confirmed at BJHS (Design & Modeling, Automation & Robotics, Medical Detectives)
- Board meetings indexed (2025-present calendar)
- Science curriculum gap identified — no confirmed publisher (white space)
- 5 vendors/partners mapped with competitive analysis
- Entry strategy targeting Instructional Services Director + Mac Robertson (PLTW champion)
- Budget pathway: Title IV-A (SSAE) + LCFF Supplemental ($9.3M)
- CDE Priority Score: 95/100 | CAST 11.37% | Math 13.29% | EL science 3.28%

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/comparison.xlsx
+++ b/comparison.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q16"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1762,6 +1762,87 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Beardsley Elementary School District</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Kern</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>1946</v>
+      </c>
+      <c r="D17" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>K-8 (TK-8)</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Paul Miller</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>17369</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>~$37-41M</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>20:1</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>63.6%</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>6.0%</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>25.2%</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>~1%</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>40%+ (CEP)</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>12.8% (249 students)</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>N/A (K-8)</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>2/10</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:Q1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1774,7 +1855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2751,6 +2832,66 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Beardsley Elementary School District</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>TBD (no confirmed publisher)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>N/A (K-8 only)</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>$9,345,675 (LCAP 2025-26 projection)</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>TBD (CEP district)</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>$50-150K (est.)</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>PLTW Gateway (D&amp;M, A&amp;R, Medical Det.) at BJHS; ASES; Science Fair; Boys &amp; Girls Club</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2763,7 +2904,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I69"/>
+  <dimension ref="A1:I74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5884,6 +6025,231 @@
         <v>5</v>
       </c>
     </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Beardsley Elementary School District</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>[Director of Instructional Services - TBD]</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Director of Instructional Services</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>instserv@beardsley.k12.ca.us</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>(661) 393-3077</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Instructional Services</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Curriculum/EdTech decision maker</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Beardsley Elementary School District</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Mac Robertson</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>PLTW Teacher + RTI Math, BJHS</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>mrobertson@beardsley.k12.ca.us</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>(661) 392-9254</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>BJHS</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Internal champion; PLTW + RTI Math</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Beardsley Elementary School District</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Ryan Frank</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Director of Technology</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>rfrank@beardsley.k12.ca.us</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>(661) 393-8550</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>EdTech integration; Clever/PowerSchool</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Potential</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Beardsley Elementary School District</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Jack Chen</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Assistant Superintendent</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>jachen@beardsley.k12.ca.us</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>(661) 393-8550</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>District Office</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Executive approval; budget authority</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Beardsley Elementary School District</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Paul Miller</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Superintendent</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>pamiller@beardsley.k12.ca.us</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>(661) 393-8550</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>District Office</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Final decision maker (since 2012)</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5896,7 +6262,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6067,6 +6433,58 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Beardsley Elementary School District</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>PLTW contract renewal (est.)</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>STEM/Curriculum</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Title IV-A</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>PLTW</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Board page: beardsleyschool.org</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>PLTW Gateway active at BJHS; annual license expected</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6079,7 +6497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I103"/>
+  <dimension ref="A1:I108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10849,6 +11267,241 @@
         </is>
       </c>
     </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Beardsley Elementary School District</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>PLTW (Project Lead The Way)</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>STEM Curriculum</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Gateway Middle School courses: Design &amp; Modeling, Automation &amp; Robotics, Medical Detectives</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Complementary (ALLY)</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>Active partnership</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>Mac Robertson is PLTW teacher; active at BJHS grades 7-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Beardsley Elementary School District</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Clever</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Student SSO Portal</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Not competitive</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Confirmed active</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>ModelIt integrates via Clever - zero new login for students</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Beardsley Elementary School District</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>PowerSchool</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Technology (SIS)</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Student Information System</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Not competitive</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Confirmed active</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>Standard SIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Beardsley Elementary School District</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Boys &amp; Girls Club of Kern County</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Community Partner</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>After-school enrichment</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Not competitive</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Active partnership</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>After-school delivery vehicle for ModelIt pilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Beardsley Elementary School District</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>[Core science publisher - UNKNOWN]</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Curriculum</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>K-8 science</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Potentially competitive</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>White space</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>NO confirmed science publisher - greenfield opportunity</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10861,7 +11514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13178,6 +13831,100 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Beardsley Elementary School District</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>K-5</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>No confirmed science curriculum - white space for ModelIt</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Beardsley Elementary School District</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>6-8</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>UNKNOWN</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>Core science unknown; PLTW elective confirmed (Design &amp; Modeling, Automation &amp; Robotics, Medical Detectives)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:I1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -13190,7 +13937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14027,6 +14774,58 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Beardsley Elementary School District</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Instructional Services Director (TBD) via instserv@beardsley.k12.ca.us</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>BJHS PLTW + ModelIt = CAST science gap solution (11.37% CAST, 3.28% EL, PLTW already present)</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Title IV-A (SSAE) / LCFF Supplemental</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>$50-150K Title IV-A; $9.3M LCFF Supp pool</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>March 2026 outreach; June 2026 LCAP adoption</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Call (661) 393-3077 to identify Instructional Services Director; send Wave 1 emails</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>March 2026</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>PLTW champion Mac Robertson is key internal ally; CEP district with Title IV-A pathway</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:J1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -14039,7 +14838,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14976,6 +15775,64 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Beardsley Elementary School District</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>1 - Identified</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>[Instructional Services Director - TBD]</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>instserv@beardsley.k12.ca.us</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Research complete</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Call (661) 393-3077; send Wave 1 emails</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>6000</v>
+      </c>
+      <c r="J17" t="n">
+        <v>20000</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>20%</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>PLTW at BJHS, 11.37% CAST, 3.28% EL science, no confirmed science publisher, Clever integration ready, CDE priority 95/100</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add Beardsley Elementary SD district intelligence profile
- Full profile: 2,290 students, K-8, Kern County, CDS 15-63339-0000000
- 27 contacts identified; 9 verified emails from district website
- Primary entry: Tammy Barrera (Asst. Supt.) + Mac Robertson (PLTW champion)
- Board meetings indexed Aug 2025–Mar 2026 with extraction template
- Science curriculum mapped: PLTW at BJHS; K-8 science = greenfield (no incumbent)
- 7 vendors/partners identified; Clever SSO deployed (zero IT lift)
- Entry strategy: free 6-week BJHS pilot → LCAP inclusion June 2026
- Budget pathway: LCAP Supplemental/Conc. + Title IV-A
- Key hook: 8.47% Gr7 math + PLTW complement + Clever = instant pilot
- CDE priority score 95/100

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/comparison.xlsx
+++ b/comparison.xlsx
@@ -1774,14 +1774,14 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1946</v>
+        <v>2290</v>
       </c>
       <c r="D17" t="n">
         <v>4</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>K-8 (TK-8)</t>
+          <t>TK-8</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1792,54 +1792,40 @@
       <c r="G17" t="n">
         <v>17369</v>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>~$37-41M</t>
-        </is>
+      <c r="H17" t="n">
+        <v>41305758</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>20:1</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>63.6%</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>6.0%</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>25.2%</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>~1%</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>40%+ (CEP)</t>
-        </is>
-      </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>12.8% (249 students)</t>
-        </is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="K17" t="n">
+        <v>6</v>
+      </c>
+      <c r="L17" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="N17" t="n">
+        <v>16.5</v>
+      </c>
+      <c r="O17" t="n">
+        <v>1.6</v>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>N/A (K-8)</t>
+          <t>N/A - K-8 district</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>2/10</t>
+          <t>95/100 CDE Priority</t>
         </is>
       </c>
     </row>
@@ -2840,12 +2826,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBD (est. $50-150K)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>TBD (no confirmed publisher)</t>
+          <t>TBD - no confirmed publisher (greenfield)</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2860,27 +2846,27 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>~$50-150K (Title II + LCAP)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>N/A (K-8 only)</t>
+          <t>N/A - K-8 district</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>$9,345,675 (LCAP 2025-26 projection)</t>
+          <t>~$4-15M LCAP supp/conc est.</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>TBD (CEP district)</t>
+          <t>~$1-2M est.</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>$50-150K (est.)</t>
+          <t>~$5-20K (Title IV-A)</t>
         </is>
       </c>
       <c r="K17" t="n">
@@ -2888,7 +2874,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>PLTW Gateway (D&amp;M, A&amp;R, Medical Det.) at BJHS; ASES; Science Fair; Boys &amp; Girls Club</t>
+          <t>PLTW at BJHS (7-8); ASES/IMPACT after-school</t>
         </is>
       </c>
     </row>
@@ -6033,41 +6019,43 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>[Director of Instructional Services - TBD]</t>
+          <t>Tammy Barrera</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Director of Instructional Services</t>
+          <t>Assistant Superintendent (Curriculum &amp; Instruction)</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>instserv@beardsley.k12.ca.us</t>
+          <t>tbarrera@beardsley.k12.ca.us</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>(661) 393-3077</t>
+          <t>(661) 393-8550</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Instructional Services</t>
+          <t>District Office</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>Curriculum/EdTech decision maker</t>
+          <t>Primary curriculum authority; LCAP lead</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="I70" t="n">
-        <v>1</v>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>1 - Primary</t>
+        </is>
       </c>
     </row>
     <row r="71">
@@ -6083,7 +6071,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>PLTW Teacher + RTI Math, BJHS</t>
+          <t>PLTW Instructor / RTI Math (BJHS)</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -6098,12 +6086,12 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>BJHS</t>
+          <t>Beardsley JH</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>Internal champion; PLTW + RTI Math</t>
+          <t>STEM champion; models already in class</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -6111,8 +6099,10 @@
           <t>Yes</t>
         </is>
       </c>
-      <c r="I71" t="n">
-        <v>2</v>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>1 - Primary</t>
+        </is>
       </c>
     </row>
     <row r="72">
@@ -6148,16 +6138,18 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>EdTech integration; Clever/PowerSchool</t>
+          <t>Controls Clever SSO; platform approvals</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Potential</t>
-        </is>
-      </c>
-      <c r="I72" t="n">
-        <v>3</v>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>2 - Technical</t>
+        </is>
       </c>
     </row>
     <row r="73">
@@ -6168,17 +6160,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Jack Chen</t>
+          <t>Paul Miller</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Assistant Superintendent</t>
+          <t>Superintendent</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>jachen@beardsley.k12.ca.us</t>
+          <t>pamiller@beardsley.k12.ca.us</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -6193,7 +6185,7 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>Executive approval; budget authority</t>
+          <t>Final contract authority</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -6201,8 +6193,10 @@
           <t>No</t>
         </is>
       </c>
-      <c r="I73" t="n">
-        <v>4</v>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>3 - Executive</t>
+        </is>
       </c>
     </row>
     <row r="74">
@@ -6213,32 +6207,32 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Paul Miller</t>
+          <t>Monica West</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Superintendent</t>
+          <t>Principal, Beardsley Junior High</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>pamiller@beardsley.k12.ca.us</t>
+          <t>mwest@beardsley.k12.ca.us</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>(661) 393-8550</t>
+          <t>(661) 392-9254</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>District Office</t>
+          <t>BJHS</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Final decision maker (since 2012)</t>
+          <t>Pilot school decision-maker</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -6246,8 +6240,10 @@
           <t>No</t>
         </is>
       </c>
-      <c r="I74" t="n">
-        <v>5</v>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>2 - School Lead</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -6441,7 +6437,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>TBD - PDF review needed</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -6461,12 +6457,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Title IV-A</t>
+          <t>Title IV-A / General Fund</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>PLTW</t>
+          <t>Project Lead the Way (PLTW)</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -6476,12 +6472,12 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Board page: beardsleyschool.org</t>
+          <t>https://www.beardsleyschool.org/apps/pages/index.jsp?uREC_ID=3558648&amp;type=d&amp;pREC_ID=2401331</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>PLTW Gateway active at BJHS; annual license expected</t>
+          <t>PLTW active at BJHS; need board minutes to confirm contract value</t>
         </is>
       </c>
     </row>
@@ -6497,7 +6493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I108"/>
+  <dimension ref="A1:I110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11275,17 +11271,17 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>PLTW (Project Lead The Way)</t>
+          <t>Project Lead the Way (PLTW)</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>STEM Curriculum</t>
+          <t>Curriculum - STEM</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Gateway Middle School courses: Design &amp; Modeling, Automation &amp; Robotics, Medical Detectives</t>
+          <t>Design &amp; Modeling; Automation &amp; Robotics; Medical Detectives (Gr 7-8)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -11295,22 +11291,22 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Annual</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>Complementary (ALLY)</t>
+          <t>No - complementary</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>Active partnership</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>Mac Robertson is PLTW teacher; active at BJHS grades 7-8</t>
+          <t>Only confirmed curriculum vendor; natural ModelIt complement</t>
         </is>
       </c>
     </row>
@@ -11327,37 +11323,37 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Technology</t>
+          <t>Technology - SSO</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Student SSO Portal</t>
+          <t>Student/staff single sign-on portal</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Unknown (subscription)</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>Annual</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>Not competitive</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>Confirmed active</t>
+          <t>Deep integration</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>ModelIt integrates via Clever - zero new login for students</t>
+          <t>Deployed district-wide; ModelIt integrates with Clever</t>
         </is>
       </c>
     </row>
@@ -11374,37 +11370,37 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Technology (SIS)</t>
+          <t>Technology - SIS</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Student Information System</t>
+          <t>Student information system + parent portal</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>Annual</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
         <is>
-          <t>Not competitive</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H106" t="inlineStr">
         <is>
-          <t>Confirmed active</t>
+          <t>Deep integration</t>
         </is>
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>Standard SIS</t>
+          <t>District SIS; roster sync via Clever</t>
         </is>
       </c>
     </row>
@@ -11426,32 +11422,32 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>After-school enrichment</t>
+          <t>ASES/IMPACT after-school program at all 4 schools</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>ASES grant funded</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>Ongoing</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
         <is>
-          <t>Not competitive</t>
+          <t>No</t>
         </is>
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>Active partnership</t>
+          <t>Program partner</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>After-school delivery vehicle for ModelIt pilot</t>
+          <t>Free after-school for TK-8; potential ModelIt enrichment delivery channel</t>
         </is>
       </c>
     </row>
@@ -11463,17 +11459,17 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>[Core science publisher - UNKNOWN]</t>
+          <t>Fresno State (CSU Fresno)</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Curriculum</t>
+          <t>University Partner</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>K-8 science</t>
+          <t>Parent University - digital/financial literacy via Zoom</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
@@ -11483,22 +11479,116 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>Program partner</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>Bilingual program; shows district values family engagement</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Beardsley Elementary School District</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>K-8 Science Publisher (UNKNOWN)</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Curriculum - Science</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>K-8 science instruction</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr">
-        <is>
-          <t>Potentially competitive</t>
-        </is>
-      </c>
-      <c r="H108" t="inlineStr">
-        <is>
-          <t>White space</t>
-        </is>
-      </c>
-      <c r="I108" t="inlineStr">
-        <is>
-          <t>NO confirmed science publisher - greenfield opportunity</t>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>GREENFIELD - no confirmed publisher; ModelIt enters white space</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Beardsley Elementary School District</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Math Publisher (UNKNOWN)</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Curriculum - Math</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>K-8 math instruction</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>Not confirmed; RTI Math noted at BJHS</t>
         </is>
       </c>
     </row>
@@ -11514,7 +11604,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13839,7 +13929,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>K-5</t>
+          <t>TK-3</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -13849,32 +13939,32 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
+          <t>Textbook (TBD)</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>No confirmed science curriculum - white space for ModelIt</t>
+          <t>No confirmed publisher; SARC review needed</t>
         </is>
       </c>
     </row>
@@ -13886,7 +13976,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>6-8</t>
+          <t>4-6</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -13896,32 +13986,79 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
+          <t>Textbook (TBD)</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Core science unknown; PLTW elective confirmed (Design &amp; Modeling, Automation &amp; Robotics, Medical Detectives)</t>
+          <t>CAST at Grade 5; critical grade band; greenfield for ModelIt</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Beardsley Elementary School District</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>7-8</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>PLTW (partial) + traditional science</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>STEM program + textbook</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Partial (PLTW NGSS-aligned)</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>PLTW confirmed; textbook publisher unknown; SEP-2 gap exists</t>
         </is>
       </c>
     </row>
@@ -14782,27 +14919,27 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Instructional Services Director (TBD) via instserv@beardsley.k12.ca.us</t>
+          <t>Tammy Barrera (tbarrera@beardsley.k12.ca.us) / Mac Robertson (mrobertson@beardsley.k12.ca.us)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>BJHS PLTW + ModelIt = CAST science gap solution (11.37% CAST, 3.28% EL, PLTW already present)</t>
+          <t>BJHS 7th grade math 8.47% + PLTW complement + Clever SSO deployed = free 6-week pilot with zero IT lift</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Title IV-A (SSAE) / LCFF Supplemental</t>
+          <t>LCAP Supplemental/Conc Grant + Title IV-A</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>$50-150K Title IV-A; $9.3M LCFF Supp pool</t>
+          <t>$50-150K LCAP; $5-20K Title IV-A</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>March 2026 outreach; June 2026 LCAP adoption</t>
+          <t>March 2026 outreach → May-June 2026 free pilot → June 2026 LCAP inclusion → Sep 2026 paid contract</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -14812,7 +14949,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Call (661) 393-3077 to identify Instructional Services Director; send Wave 1 emails</t>
+          <t>Email Barrera + Robertson + Frank; offer free 6-week BJHS pilot</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -14822,7 +14959,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>PLTW champion Mac Robertson is key internal ally; CEP district with Title IV-A pathway</t>
+          <t>Greenfield science publisher; PLTW at JH; Clever SSO in place; 13.29% math / 11.37% science; 95/100 CDE priority</t>
         </is>
       </c>
     </row>
@@ -15788,17 +15925,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>[Instructional Services Director - TBD]</t>
+          <t>Tammy Barrera</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>instserv@beardsley.k12.ca.us</t>
+          <t>tbarrera@beardsley.k12.ca.us</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Research complete</t>
+          <t>Research complete; profile built</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -15808,28 +15945,32 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Call (661) 393-3077; send Wave 1 emails</t>
+          <t>Send intro email to Barrera + Robertson + Frank</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2026-03-09</t>
-        </is>
-      </c>
-      <c r="I17" t="n">
-        <v>6000</v>
-      </c>
-      <c r="J17" t="n">
-        <v>20000</v>
+          <t>March 2026</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>$12-20K pilot</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>$35-60K district-wide</t>
+        </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>20%</t>
+          <t>Medium-High</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>PLTW at BJHS, 11.37% CAST, 3.28% EL science, no confirmed science publisher, Clever integration ready, CDE priority 95/100</t>
+          <t>PLTW champion (Robertson) in place; Clever deployed; greenfield science; 8.47% Gr7 math; 95/100 CDE priority</t>
         </is>
       </c>
     </row>

</xml_diff>